<commit_message>
#3 Main-Board & Termination-Board PCB Updated, Deliverables updated
</commit_message>
<xml_diff>
--- a/Design-Files/Main-Controller-Board-v1.1.0/Deliverables/BOM/Client_BOM_Main-Controller-Board-v1.1.0.xlsx
+++ b/Design-Files/Main-Controller-Board-v1.1.0/Deliverables/BOM/Client_BOM_Main-Controller-Board-v1.1.0.xlsx
@@ -5,7 +5,7 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\benjamin-rcctledboard-hw\Design-Files\Main-Controller-Board-v1.0.0\Project Outputs for Main-Controller-Board-v1.0.0\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\benjamin-rcctledboard-hw\Design-Files\Main-Controller-Board-v1.1.0\Deliverables\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="242" uniqueCount="177">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="242" uniqueCount="179">
   <si>
     <t>#</t>
   </si>
@@ -30,6 +30,9 @@
     <t>Capacitor</t>
   </si>
   <si>
+    <t>Capacitors</t>
+  </si>
+  <si>
     <t>Diode</t>
   </si>
   <si>
@@ -48,7 +51,7 @@
     <t>Transistors</t>
   </si>
   <si>
-    <t>MOSFET</t>
+    <t>MOSFETs</t>
   </si>
   <si>
     <t>Resistors</t>
@@ -105,7 +108,7 @@
     <t>D2</t>
   </si>
   <si>
-    <t>F1, F3</t>
+    <t>F1, F2</t>
   </si>
   <si>
     <t>J1</t>
@@ -201,22 +204,22 @@
     <t>CAP CER 10UF 25V X7R 1210</t>
   </si>
   <si>
-    <t>DIODE SCHOTTKY 60V 2A SMA</t>
+    <t>SCHOTTKY DIODE SMB 100V 5A</t>
   </si>
   <si>
     <t>SMB(DO-214AA) TVS ROHS</t>
   </si>
   <si>
-    <t>33V 1.1A 40A 2.2A 1812 Resettable Fuses ROHS</t>
-  </si>
-  <si>
-    <t>CONN PWR JACK 2X5.5MM SOLDER</t>
+    <t>30V 3.3A 40A 6.6A 2920 Resettable Fuses ROHS</t>
+  </si>
+  <si>
+    <t>Bend insert DC Power Receptacle -20℃~+70℃ 1.3mm 5mm 3.5A 24V Plugin DC Power Connectors ROHS</t>
   </si>
   <si>
     <t>1x6P SH 1 1mm 6 SMD,P=1mm Wire To Board / Wire To Wire Connector ROHS</t>
   </si>
   <si>
-    <t>CONN HEADER SMD R/A 5POS 2MM</t>
+    <t>CONN HEADER R/A 5POS 2.5MM</t>
   </si>
   <si>
     <t>2.26A 4.7uH ±20% SMD,7.3x7.3mm Power Inductors ROHS</t>
@@ -231,7 +234,7 @@
     <t>65V 200mW 220@2mA,5V 100mA PNP SOT-23 Bipolar Transistors - BJT ROHS</t>
   </si>
   <si>
-    <t>MOSFET N-CH 55V 5.5A SOT223</t>
+    <t>MOSFET N-CH 55V 12A SOT223</t>
   </si>
   <si>
     <t>RES 0 OHM JUMPER 1/16W 0402</t>
@@ -291,13 +294,13 @@
     <t>189RV0019</t>
   </si>
   <si>
-    <t>SMA</t>
-  </si>
-  <si>
-    <t>PJ-051AH</t>
-  </si>
-  <si>
-    <t>S5B-PH-SM4-TB(LF)(SN)</t>
+    <t>Fuse-2920</t>
+  </si>
+  <si>
+    <t>DC-003A-3.5A-1.3</t>
+  </si>
+  <si>
+    <t>S5B-XH-A(LF)(SN)</t>
   </si>
   <si>
     <t>YPRH0703-4R7M</t>
@@ -360,13 +363,13 @@
     <t>C3225X7R1E106M250AC</t>
   </si>
   <si>
-    <t>B260A-13-F</t>
+    <t>SS510B</t>
   </si>
   <si>
     <t>SMBJ26CA</t>
   </si>
   <si>
-    <t>BSMD1812-110-33V</t>
+    <t>BSMD2920-330-30V</t>
   </si>
   <si>
     <t>C145963</t>
@@ -381,7 +384,7 @@
     <t>BC856B</t>
   </si>
   <si>
-    <t>BUK98150-55A/CUF</t>
+    <t>BUK9832-55A/CUX</t>
   </si>
   <si>
     <t>RC0402FR-070RL</t>
@@ -432,30 +435,33 @@
     <t>TDK Corporation</t>
   </si>
   <si>
+    <t>MDD</t>
+  </si>
+  <si>
+    <t>MSKSEMI</t>
+  </si>
+  <si>
+    <t>BHFUSE</t>
+  </si>
+  <si>
+    <t>XKB Connection</t>
+  </si>
+  <si>
+    <t>BOOMELE</t>
+  </si>
+  <si>
+    <t>JST</t>
+  </si>
+  <si>
+    <t>YJYCOIN</t>
+  </si>
+  <si>
+    <t>Foshan NationStar Optoelectronics</t>
+  </si>
+  <si>
     <t>Diodes</t>
   </si>
   <si>
-    <t>MSKSEMI</t>
-  </si>
-  <si>
-    <t>BHFUSE</t>
-  </si>
-  <si>
-    <t>CUI Devices</t>
-  </si>
-  <si>
-    <t>BOOMELE</t>
-  </si>
-  <si>
-    <t>JST</t>
-  </si>
-  <si>
-    <t>YJYCOIN</t>
-  </si>
-  <si>
-    <t>Foshan NationStar Optoelectronics</t>
-  </si>
-  <si>
     <t>Guangdong Hottech</t>
   </si>
   <si>
@@ -531,22 +537,22 @@
     <t>Value</t>
   </si>
   <si>
+    <t>https://fr.aliexpress.com/item/1005004709078383.html?spm=a2g0o.productlist.main.57.6d95f397cf7gmb&amp;algo_pvid=edcdcb7e-db68-42b8-a831-237760419952&amp;algo_exp_id=edcdcb7e-db68-42b8-a831-237760419952-</t>
+  </si>
+  <si>
     <t>Module</t>
   </si>
   <si>
+    <t>51R 1W (Custom)</t>
+  </si>
+  <si>
     <t>-</t>
   </si>
   <si>
-    <t>Fuse-1812</t>
-  </si>
-  <si>
     <t>Custom</t>
   </si>
   <si>
-    <t>https://fr.aliexpress.com/item/1005004709078383.html?spm=a2g0o.productlist.main.57.6d95f397cf7gmb&amp;algo_pvid=edcdcb7e-db68-42b8-a831-237760419952&amp;algo_exp_id=edcdcb7e-db68-42b8-a831-237760419952-28&amp;pdp_npi=4%40dis%21USD%211.74%211.13%21%21%211.74%21%21%40210321dc17013352231813956e2690%2112000030183281143%21sea%21FR%210%21AB&amp;curPageLogUid=DS5ZvT9x3Or6</t>
-  </si>
-  <si>
-    <t>51R 1W (Custom)</t>
+    <t>SMB</t>
   </si>
   <si>
     <t>SMB (DO-214AA)</t>
@@ -1067,7 +1073,7 @@
     <col min="8" max="8" width="21.42578125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="17.85546875" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="16.7109375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="29.28515625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="29.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1092,28 +1098,28 @@
         <v>1</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="I2" s="6" t="s">
+        <v>171</v>
+      </c>
+      <c r="J2" s="5" t="s">
         <v>169</v>
       </c>
-      <c r="J2" s="5" t="s">
-        <v>167</v>
-      </c>
       <c r="K2" s="5" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
     </row>
     <row r="3" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1126,22 +1132,22 @@
         <v>2</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="H3" s="7" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="I3" s="8" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="J3" s="7">
         <v>2</v>
@@ -1158,22 +1164,22 @@
         <v>2</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E4" s="10" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="G4" s="10" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="I4" s="10" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="J4" s="9">
         <v>2</v>
@@ -1190,22 +1196,22 @@
         <v>2</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="H5" s="7" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="I5" s="8" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="J5" s="7">
         <v>3</v>
@@ -1222,22 +1228,22 @@
         <v>2</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E6" s="10" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="F6" s="9" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="G6" s="10" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="H6" s="9" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="I6" s="10" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="J6" s="9">
         <v>1</v>
@@ -1250,26 +1256,26 @@
         <f>ROW(B7) - ROW($B$2)</f>
         <v>5</v>
       </c>
-      <c r="C7" s="13" t="s">
+      <c r="C7" s="12" t="s">
         <v>2</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="H7" s="7" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="I7" s="8" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="J7" s="7">
         <v>1</v>
@@ -1286,22 +1292,22 @@
         <v>2</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="F8" s="9" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="G8" s="10" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="H8" s="9" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="I8" s="10" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="J8" s="9">
         <v>1</v>
@@ -1318,22 +1324,22 @@
         <v>2</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="H9" s="7" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="I9" s="8" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="J9" s="7">
         <v>1</v>
@@ -1350,22 +1356,22 @@
         <v>2</v>
       </c>
       <c r="D10" s="9" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="F10" s="9" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="G10" s="10" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="H10" s="9" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="I10" s="10" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="J10" s="9">
         <v>3</v>
@@ -1379,25 +1385,25 @@
         <v>9</v>
       </c>
       <c r="C11" s="12" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="G11" s="8" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="H11" s="7" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="I11" s="8" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="J11" s="7">
         <v>3</v>
@@ -1411,25 +1417,25 @@
         <v>10</v>
       </c>
       <c r="C12" s="13" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E12" s="10" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F12" s="9" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="G12" s="10" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="H12" s="9" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="I12" s="10" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="J12" s="9">
         <v>1</v>
@@ -1443,25 +1449,25 @@
         <v>11</v>
       </c>
       <c r="C13" s="12" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>90</v>
+        <v>177</v>
       </c>
       <c r="G13" s="8" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="H13" s="7" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="I13" s="8" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
       <c r="J13" s="7">
         <v>1</v>
@@ -1475,25 +1481,25 @@
         <v>12</v>
       </c>
       <c r="C14" s="13" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D14" s="9" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E14" s="10" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="F14" s="9" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="G14" s="10" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="H14" s="9" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="I14" s="10" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
       <c r="J14" s="9">
         <v>1</v>
@@ -1507,57 +1513,57 @@
         <v>13</v>
       </c>
       <c r="C15" s="12" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D15" s="7" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E15" s="8" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="F15" s="7" t="s">
-        <v>172</v>
+        <v>91</v>
       </c>
       <c r="G15" s="8" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="H15" s="7" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="I15" s="8" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
       <c r="J15" s="7">
         <v>2</v>
       </c>
       <c r="K15" s="7"/>
     </row>
-    <row r="16" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="1"/>
       <c r="B16" s="11">
         <f t="shared" si="0"/>
         <v>14</v>
       </c>
       <c r="C16" s="13" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D16" s="9" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E16" s="10" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="F16" s="9" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="G16" s="10" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="H16" s="9" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="I16" s="10" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
       <c r="J16" s="9">
         <v>1</v>
@@ -1571,25 +1577,25 @@
         <v>15</v>
       </c>
       <c r="C17" s="12" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D17" s="7" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E17" s="8" t="s">
-        <v>64</v>
-      </c>
-      <c r="F17" s="7" t="s">
-        <v>173</v>
+        <v>65</v>
+      </c>
+      <c r="F17" s="9" t="s">
+        <v>176</v>
       </c>
       <c r="G17" s="8" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="H17" s="7" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="I17" s="8" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
       <c r="J17" s="7">
         <v>2</v>
@@ -1603,25 +1609,25 @@
         <v>16</v>
       </c>
       <c r="C18" s="12" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D18" s="9" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="E18" s="10" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F18" s="9" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="G18" s="10" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="H18" s="9" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="I18" s="10" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
       <c r="J18" s="9">
         <v>1</v>
@@ -1635,25 +1641,25 @@
         <v>17</v>
       </c>
       <c r="C19" s="12" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D19" s="7" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E19" s="8" t="s">
-        <v>66</v>
-      </c>
-      <c r="F19" s="7" t="s">
-        <v>173</v>
+        <v>67</v>
+      </c>
+      <c r="F19" s="9" t="s">
+        <v>176</v>
       </c>
       <c r="G19" s="8" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="H19" s="7" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="I19" s="8" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="J19" s="7">
         <v>1</v>
@@ -1667,25 +1673,25 @@
         <v>18</v>
       </c>
       <c r="C20" s="13" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D20" s="9" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E20" s="10" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F20" s="9" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="G20" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="H20" s="9" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="I20" s="10" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
       <c r="J20" s="9">
         <v>1</v>
@@ -1699,25 +1705,25 @@
         <v>19</v>
       </c>
       <c r="C21" s="12" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D21" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E21" s="8" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="F21" s="7" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="G21" s="8" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="H21" s="7" t="s">
-        <v>137</v>
+        <v>146</v>
       </c>
       <c r="I21" s="8" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
       <c r="J21" s="7">
         <v>6</v>
@@ -1731,25 +1737,25 @@
         <v>20</v>
       </c>
       <c r="C22" s="13" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D22" s="9" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E22" s="10" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="F22" s="9" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="G22" s="10" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="H22" s="9" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="I22" s="10" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
       <c r="J22" s="9">
         <v>3</v>
@@ -1763,25 +1769,25 @@
         <v>21</v>
       </c>
       <c r="C23" s="12" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D23" s="7" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E23" s="8" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="F23" s="7" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="G23" s="8" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="H23" s="7" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="I23" s="8" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
       <c r="J23" s="7">
         <v>3</v>
@@ -1795,25 +1801,25 @@
         <v>22</v>
       </c>
       <c r="C24" s="13" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D24" s="9" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="E24" s="10" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="F24" s="9" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="G24" s="10" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="H24" s="9" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="I24" s="10" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="J24" s="9">
         <v>2</v>
@@ -1827,25 +1833,25 @@
         <v>23</v>
       </c>
       <c r="C25" s="13" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D25" s="7" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="E25" s="8" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="F25" s="7" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="G25" s="8" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="H25" s="7" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="I25" s="8" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="J25" s="7">
         <v>4</v>
@@ -1859,25 +1865,25 @@
         <v>24</v>
       </c>
       <c r="C26" s="13" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D26" s="9" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E26" s="10" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="F26" s="9" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="G26" s="10" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="H26" s="9" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="I26" s="10" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="J26" s="9">
         <v>1</v>
@@ -1891,25 +1897,25 @@
         <v>25</v>
       </c>
       <c r="C27" s="12" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D27" s="7" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="E27" s="8" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="F27" s="7" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="G27" s="8" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="H27" s="7" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="I27" s="8" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="J27" s="7">
         <v>1</v>
@@ -1923,63 +1929,63 @@
         <v>26</v>
       </c>
       <c r="C28" s="13" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D28" s="9" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E28" s="10" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F28" s="9" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="G28" s="10" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="H28" s="9" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="I28" s="10" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="J28" s="9">
         <v>6</v>
       </c>
       <c r="K28" s="9"/>
     </row>
-    <row r="29" spans="1:11" ht="225.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:11" ht="120.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="1"/>
       <c r="B29" s="11">
         <f>ROW(B29) - ROW($B$2)</f>
         <v>27</v>
       </c>
       <c r="C29" s="12" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D29" s="7" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="E29" s="8" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="F29" s="7" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="G29" s="8" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="H29" s="7" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="I29" s="8" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="J29" s="7">
         <v>3</v>
       </c>
       <c r="K29" s="15" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
     </row>
     <row r="30" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1989,25 +1995,25 @@
         <v>28</v>
       </c>
       <c r="C30" s="13" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D30" s="9" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="E30" s="10" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="F30" s="9" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="G30" s="10" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="H30" s="9" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="I30" s="10" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="J30" s="9">
         <v>3</v>
@@ -2021,25 +2027,25 @@
         <v>29</v>
       </c>
       <c r="C31" s="12" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D31" s="7" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E31" s="8" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="F31" s="7" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="G31" s="8" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="H31" s="7" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="I31" s="8" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
       <c r="J31" s="7">
         <v>2</v>
@@ -2053,25 +2059,25 @@
         <v>30</v>
       </c>
       <c r="C32" s="13" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D32" s="9" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E32" s="10" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="F32" s="9" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="G32" s="10" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="H32" s="9" t="s">
-        <v>137</v>
+        <v>146</v>
       </c>
       <c r="I32" s="10" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
       <c r="J32" s="9">
         <v>1</v>
@@ -2085,25 +2091,25 @@
         <v>31</v>
       </c>
       <c r="C33" s="12" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D33" s="7" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="E33" s="8" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="F33" s="7" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="G33" s="8" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="H33" s="7" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="I33" s="8" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
       <c r="J33" s="7">
         <v>1</v>
@@ -2117,25 +2123,25 @@
         <v>32</v>
       </c>
       <c r="C34" s="13" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="D34" s="9" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E34" s="10" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F34" s="9" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="G34" s="10" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="H34" s="9" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="I34" s="10" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
       <c r="J34" s="9">
         <v>1</v>
@@ -2149,25 +2155,25 @@
         <v>33</v>
       </c>
       <c r="C35" s="12" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D35" s="7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="E35" s="8" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="F35" s="7" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="G35" s="8" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="H35" s="7" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="I35" s="8" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
       <c r="J35" s="7">
         <v>3</v>
@@ -2179,9 +2185,9 @@
     <mergeCell ref="I1:K1"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="K29"/>
+    <hyperlink ref="K29" r:id="rId1"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
#3 0.1uF CAP Part No. updated in BOM
</commit_message>
<xml_diff>
--- a/Design-Files/Main-Controller-Board-v1.1.0/Deliverables/BOM/Client_BOM_Main-Controller-Board-v1.1.0.xlsx
+++ b/Design-Files/Main-Controller-Board-v1.1.0/Deliverables/BOM/Client_BOM_Main-Controller-Board-v1.1.0.xlsx
@@ -5,7 +5,7 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\benjamin-rcctledboard-hw\Design-Files\Main-Controller-Board-v1.1.0\Deliverables\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-consultants\benjamin-rcctledboard-hw\Design-Files\Main-Controller-Board-v1.1.0\Deliverables\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -183,9 +183,6 @@
     <t>CAP CER 22UF 10V X5R 0805</t>
   </si>
   <si>
-    <t>CAP CER 0.1UF 25V X7R 0603</t>
-  </si>
-  <si>
     <t>CAP CER 1UF 100V X7S 0805</t>
   </si>
   <si>
@@ -345,9 +342,6 @@
     <t>GRM21BR61A226ME44L</t>
   </si>
   <si>
-    <t>CC0603JRX7R8BB104</t>
-  </si>
-  <si>
     <t>GCM21BC72A105KE36L</t>
   </si>
   <si>
@@ -556,6 +550,12 @@
   </si>
   <si>
     <t>SMB (DO-214AA)</t>
+  </si>
+  <si>
+    <t>CC0603JRX7R9BB104</t>
+  </si>
+  <si>
+    <t>CAP CER 0.1UF 50V X7R 0603</t>
   </si>
 </sst>
 </file>
@@ -767,11 +767,11 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="6" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="6" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1062,21 +1062,21 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:K35"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="3.140625" style="4" customWidth="1"/>
-    <col min="3" max="3" width="18.7109375" style="4" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="3.109375" style="4" customWidth="1"/>
+    <col min="3" max="3" width="18.6640625" style="4" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="36" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="30" customWidth="1"/>
-    <col min="6" max="6" width="26.5703125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="33.42578125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="21.42578125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="17.85546875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="16.7109375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="29.42578125" customWidth="1"/>
+    <col min="6" max="6" width="26.5546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="33.44140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="21.44140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="17.88671875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="16.6640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="29.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1"/>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -1085,11 +1085,11 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
-      <c r="I1" s="14"/>
-      <c r="J1" s="14"/>
-      <c r="K1" s="14"/>
-    </row>
-    <row r="2" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I1" s="15"/>
+      <c r="J1" s="15"/>
+      <c r="K1" s="15"/>
+    </row>
+    <row r="2" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="1"/>
       <c r="B2" s="5" t="s">
         <v>0</v>
@@ -1104,25 +1104,25 @@
         <v>50</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="I2" s="6" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="J2" s="5" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="K2" s="5" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="1"/>
       <c r="B3" s="11">
         <f>ROW(B3) - ROW($B$2)</f>
@@ -1138,23 +1138,23 @@
         <v>51</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="H3" s="7" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="I3" s="8" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="J3" s="7">
         <v>2</v>
       </c>
       <c r="K3" s="7"/>
     </row>
-    <row r="4" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:11" ht="36.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="1"/>
       <c r="B4" s="11">
         <f t="shared" ref="B4:B34" si="0">ROW(B4) - ROW($B$2)</f>
@@ -1170,23 +1170,23 @@
         <v>52</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="G4" s="10" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="I4" s="10" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="J4" s="9">
         <v>2</v>
       </c>
       <c r="K4" s="9"/>
     </row>
-    <row r="5" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="1"/>
       <c r="B5" s="11">
         <f>ROW(B5) - ROW($B$2)</f>
@@ -1202,23 +1202,23 @@
         <v>53</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="H5" s="7" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="I5" s="8" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="J5" s="7">
         <v>3</v>
       </c>
       <c r="K5" s="7"/>
     </row>
-    <row r="6" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" s="1"/>
       <c r="B6" s="11">
         <f t="shared" si="0"/>
@@ -1231,26 +1231,26 @@
         <v>20</v>
       </c>
       <c r="E6" s="10" t="s">
-        <v>54</v>
+        <v>178</v>
       </c>
       <c r="F6" s="9" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="G6" s="10" t="s">
-        <v>108</v>
+        <v>177</v>
       </c>
       <c r="H6" s="9" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="I6" s="10" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="J6" s="9">
         <v>1</v>
       </c>
       <c r="K6" s="9"/>
     </row>
-    <row r="7" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" s="1"/>
       <c r="B7" s="11">
         <f>ROW(B7) - ROW($B$2)</f>
@@ -1263,26 +1263,26 @@
         <v>21</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="H7" s="7" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="I7" s="8" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="J7" s="7">
         <v>1</v>
       </c>
       <c r="K7" s="7"/>
     </row>
-    <row r="8" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:11" ht="36.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A8" s="1"/>
       <c r="B8" s="11">
         <f t="shared" si="0"/>
@@ -1295,26 +1295,26 @@
         <v>22</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F8" s="9" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="G8" s="10" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="H8" s="9" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="I8" s="10" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="J8" s="9">
         <v>1</v>
       </c>
       <c r="K8" s="9"/>
     </row>
-    <row r="9" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A9" s="1"/>
       <c r="B9" s="11">
         <f>ROW(B9) - ROW($B$2)</f>
@@ -1327,26 +1327,26 @@
         <v>23</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="H9" s="7" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="I9" s="8" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="J9" s="7">
         <v>1</v>
       </c>
       <c r="K9" s="7"/>
     </row>
-    <row r="10" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A10" s="1"/>
       <c r="B10" s="11">
         <f t="shared" si="0"/>
@@ -1359,26 +1359,26 @@
         <v>24</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="F10" s="9" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="G10" s="10" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="H10" s="9" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="I10" s="10" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="J10" s="9">
         <v>3</v>
       </c>
       <c r="K10" s="9"/>
     </row>
-    <row r="11" spans="1:11" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:11" ht="48.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11" s="1"/>
       <c r="B11" s="11">
         <f>ROW(B11) - ROW($B$2)</f>
@@ -1391,26 +1391,26 @@
         <v>25</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="G11" s="8" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="H11" s="7" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="I11" s="8" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="J11" s="7">
         <v>3</v>
       </c>
       <c r="K11" s="7"/>
     </row>
-    <row r="12" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A12" s="1"/>
       <c r="B12" s="11">
         <f t="shared" si="0"/>
@@ -1423,26 +1423,26 @@
         <v>26</v>
       </c>
       <c r="E12" s="10" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F12" s="9" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="G12" s="10" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="H12" s="9" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="I12" s="10" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="J12" s="9">
         <v>1</v>
       </c>
       <c r="K12" s="9"/>
     </row>
-    <row r="13" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A13" s="1"/>
       <c r="B13" s="11">
         <f>ROW(B13) - ROW($B$2)</f>
@@ -1455,26 +1455,26 @@
         <v>27</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="G13" s="8" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="H13" s="7" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="I13" s="8" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="J13" s="7">
         <v>1</v>
       </c>
       <c r="K13" s="7"/>
     </row>
-    <row r="14" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A14" s="1"/>
       <c r="B14" s="11">
         <f t="shared" si="0"/>
@@ -1487,26 +1487,26 @@
         <v>28</v>
       </c>
       <c r="E14" s="10" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="F14" s="9" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="G14" s="10" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="H14" s="9" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="I14" s="10" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="J14" s="9">
         <v>1</v>
       </c>
       <c r="K14" s="9"/>
     </row>
-    <row r="15" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:11" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A15" s="1"/>
       <c r="B15" s="11">
         <f>ROW(B15) - ROW($B$2)</f>
@@ -1519,26 +1519,26 @@
         <v>29</v>
       </c>
       <c r="E15" s="8" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="F15" s="7" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="G15" s="8" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="H15" s="7" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="I15" s="8" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="J15" s="7">
         <v>2</v>
       </c>
       <c r="K15" s="7"/>
     </row>
-    <row r="16" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:11" ht="36.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A16" s="1"/>
       <c r="B16" s="11">
         <f t="shared" si="0"/>
@@ -1551,26 +1551,26 @@
         <v>30</v>
       </c>
       <c r="E16" s="10" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="F16" s="9" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="G16" s="10" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="H16" s="9" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="I16" s="10" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="J16" s="9">
         <v>1</v>
       </c>
       <c r="K16" s="9"/>
     </row>
-    <row r="17" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:11" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A17" s="1"/>
       <c r="B17" s="11">
         <f>ROW(B17) - ROW($B$2)</f>
@@ -1583,26 +1583,26 @@
         <v>31</v>
       </c>
       <c r="E17" s="8" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F17" s="9" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="G17" s="8" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="H17" s="7" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="I17" s="8" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="J17" s="7">
         <v>2</v>
       </c>
       <c r="K17" s="7"/>
     </row>
-    <row r="18" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A18" s="1"/>
       <c r="B18" s="11">
         <f t="shared" si="0"/>
@@ -1615,26 +1615,26 @@
         <v>32</v>
       </c>
       <c r="E18" s="10" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="F18" s="9" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="G18" s="10" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="H18" s="9" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="I18" s="10" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="J18" s="9">
         <v>1</v>
       </c>
       <c r="K18" s="9"/>
     </row>
-    <row r="19" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:11" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A19" s="1"/>
       <c r="B19" s="11">
         <f>ROW(B19) - ROW($B$2)</f>
@@ -1647,26 +1647,26 @@
         <v>33</v>
       </c>
       <c r="E19" s="8" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="F19" s="9" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="G19" s="8" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="H19" s="7" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="I19" s="8" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="J19" s="7">
         <v>1</v>
       </c>
       <c r="K19" s="7"/>
     </row>
-    <row r="20" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:11" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A20" s="1"/>
       <c r="B20" s="11">
         <f t="shared" si="0"/>
@@ -1679,26 +1679,26 @@
         <v>34</v>
       </c>
       <c r="E20" s="10" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="F20" s="9" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="G20" s="10" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="H20" s="9" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="I20" s="10" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="J20" s="9">
         <v>1</v>
       </c>
       <c r="K20" s="9"/>
     </row>
-    <row r="21" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A21" s="1"/>
       <c r="B21" s="11">
         <f>ROW(B21) - ROW($B$2)</f>
@@ -1711,26 +1711,26 @@
         <v>35</v>
       </c>
       <c r="E21" s="8" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F21" s="7" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="G21" s="8" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="H21" s="7" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="I21" s="8" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="J21" s="7">
         <v>6</v>
       </c>
       <c r="K21" s="7"/>
     </row>
-    <row r="22" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:11" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A22" s="1"/>
       <c r="B22" s="11">
         <f t="shared" si="0"/>
@@ -1743,26 +1743,26 @@
         <v>36</v>
       </c>
       <c r="E22" s="10" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F22" s="9" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="G22" s="10" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="H22" s="9" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="I22" s="10" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="J22" s="9">
         <v>3</v>
       </c>
       <c r="K22" s="9"/>
     </row>
-    <row r="23" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A23" s="1"/>
       <c r="B23" s="11">
         <f>ROW(B23) - ROW($B$2)</f>
@@ -1775,26 +1775,26 @@
         <v>37</v>
       </c>
       <c r="E23" s="8" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="F23" s="7" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="G23" s="8" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="H23" s="7" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="I23" s="8" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="J23" s="7">
         <v>3</v>
       </c>
       <c r="K23" s="7"/>
     </row>
-    <row r="24" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A24" s="1"/>
       <c r="B24" s="11">
         <f t="shared" si="0"/>
@@ -1807,26 +1807,26 @@
         <v>38</v>
       </c>
       <c r="E24" s="10" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="F24" s="9" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="G24" s="10" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="H24" s="9" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="I24" s="10" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="J24" s="9">
         <v>2</v>
       </c>
       <c r="K24" s="9"/>
     </row>
-    <row r="25" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A25" s="1"/>
       <c r="B25" s="11">
         <f>ROW(B25) - ROW($B$2)</f>
@@ -1839,26 +1839,26 @@
         <v>39</v>
       </c>
       <c r="E25" s="8" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="F25" s="7" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="G25" s="8" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="H25" s="7" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="I25" s="8" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="J25" s="7">
         <v>4</v>
       </c>
       <c r="K25" s="7"/>
     </row>
-    <row r="26" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A26" s="1"/>
       <c r="B26" s="11">
         <f t="shared" si="0"/>
@@ -1871,26 +1871,26 @@
         <v>40</v>
       </c>
       <c r="E26" s="10" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="F26" s="9" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="G26" s="10" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="H26" s="9" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="I26" s="10" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="J26" s="9">
         <v>1</v>
       </c>
       <c r="K26" s="9"/>
     </row>
-    <row r="27" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A27" s="1"/>
       <c r="B27" s="11">
         <f>ROW(B27) - ROW($B$2)</f>
@@ -1903,26 +1903,26 @@
         <v>41</v>
       </c>
       <c r="E27" s="8" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="F27" s="7" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="G27" s="8" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="H27" s="7" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="I27" s="8" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="J27" s="7">
         <v>1</v>
       </c>
       <c r="K27" s="7"/>
     </row>
-    <row r="28" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A28" s="1"/>
       <c r="B28" s="11">
         <f t="shared" si="0"/>
@@ -1935,26 +1935,26 @@
         <v>42</v>
       </c>
       <c r="E28" s="10" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="F28" s="9" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="G28" s="10" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="H28" s="9" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="I28" s="10" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="J28" s="9">
         <v>6</v>
       </c>
       <c r="K28" s="9"/>
     </row>
-    <row r="29" spans="1:11" ht="120.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:11" ht="115.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A29" s="1"/>
       <c r="B29" s="11">
         <f>ROW(B29) - ROW($B$2)</f>
@@ -1967,28 +1967,28 @@
         <v>43</v>
       </c>
       <c r="E29" s="8" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="F29" s="7" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G29" s="8" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="H29" s="7" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="I29" s="8" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="J29" s="7">
         <v>3</v>
       </c>
-      <c r="K29" s="15" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="30" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K29" s="14" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A30" s="1"/>
       <c r="B30" s="11">
         <f t="shared" si="0"/>
@@ -2001,26 +2001,26 @@
         <v>44</v>
       </c>
       <c r="E30" s="10" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="F30" s="9" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="G30" s="10" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="H30" s="9" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="I30" s="10" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="J30" s="9">
         <v>3</v>
       </c>
       <c r="K30" s="9"/>
     </row>
-    <row r="31" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A31" s="1"/>
       <c r="B31" s="11">
         <f>ROW(B31) - ROW($B$2)</f>
@@ -2033,26 +2033,26 @@
         <v>45</v>
       </c>
       <c r="E31" s="8" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F31" s="7" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="G31" s="8" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="H31" s="7" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="I31" s="8" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="J31" s="7">
         <v>2</v>
       </c>
       <c r="K31" s="7"/>
     </row>
-    <row r="32" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A32" s="1"/>
       <c r="B32" s="11">
         <f t="shared" si="0"/>
@@ -2065,26 +2065,26 @@
         <v>46</v>
       </c>
       <c r="E32" s="10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="F32" s="9" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="G32" s="10" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="H32" s="9" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="I32" s="10" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="J32" s="9">
         <v>1</v>
       </c>
       <c r="K32" s="9"/>
     </row>
-    <row r="33" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:11" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A33" s="1"/>
       <c r="B33" s="11">
         <f>ROW(B33) - ROW($B$2)</f>
@@ -2097,58 +2097,58 @@
         <v>47</v>
       </c>
       <c r="E33" s="8" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="F33" s="7" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="G33" s="8" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="H33" s="7" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="I33" s="8" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="J33" s="7">
         <v>1</v>
       </c>
       <c r="K33" s="7"/>
     </row>
-    <row r="34" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:11" ht="36.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A34" s="1"/>
       <c r="B34" s="11">
         <f t="shared" si="0"/>
         <v>32</v>
       </c>
       <c r="C34" s="13" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="D34" s="9" t="s">
         <v>48</v>
       </c>
       <c r="E34" s="10" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="F34" s="9" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="G34" s="10" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="H34" s="9" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="I34" s="10" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="J34" s="9">
         <v>1</v>
       </c>
       <c r="K34" s="9"/>
     </row>
-    <row r="35" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A35" s="1"/>
       <c r="B35" s="11">
         <f>ROW(B35) - ROW($B$2)</f>
@@ -2161,19 +2161,19 @@
         <v>49</v>
       </c>
       <c r="E35" s="8" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="F35" s="7" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="G35" s="8" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="H35" s="7" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="I35" s="8" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="J35" s="7">
         <v>3</v>

</xml_diff>

<commit_message>
#3 Termination_Board and Main_Controller_Board Schematic, PCB Updated, Deliverables Updated
</commit_message>
<xml_diff>
--- a/Design-Files/Main-Controller-Board-v1.1.0/Deliverables/BOM/Client_BOM_Main-Controller-Board-v1.1.0.xlsx
+++ b/Design-Files/Main-Controller-Board-v1.1.0/Deliverables/BOM/Client_BOM_Main-Controller-Board-v1.1.0.xlsx
@@ -5,7 +5,7 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-consultants\benjamin-rcctledboard-hw\Design-Files\Main-Controller-Board-v1.1.0\Deliverables\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\benjamin-rcctledboard-hw\Design-Files\Main-Controller-Board-v1.1.0\Deliverables\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="242" uniqueCount="179">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="242" uniqueCount="178">
   <si>
     <t>#</t>
   </si>
@@ -54,9 +54,6 @@
     <t>MOSFETs</t>
   </si>
   <si>
-    <t>Resistors</t>
-  </si>
-  <si>
     <t>Resistor</t>
   </si>
   <si>
@@ -183,6 +180,9 @@
     <t>CAP CER 22UF 10V X5R 0805</t>
   </si>
   <si>
+    <t>CAP CER 0.1UF 50V X7R 0603</t>
+  </si>
+  <si>
     <t>CAP CER 1UF 100V X7S 0805</t>
   </si>
   <si>
@@ -210,7 +210,7 @@
     <t>30V 3.3A 40A 6.6A 2920 Resettable Fuses ROHS</t>
   </si>
   <si>
-    <t>Bend insert DC Power Receptacle -20℃~+70℃ 1.3mm 5mm 3.5A 24V Plugin DC Power Connectors ROHS</t>
+    <t>Bend insert DC Power Receptacle -30℃~+85℃ 2.5mm 6mm 7A 24V Plugin DC Power Connectors ROHS</t>
   </si>
   <si>
     <t>1x6P SH 1 1mm 6 SMD,P=1mm Wire To Board / Wire To Wire Connector ROHS</t>
@@ -294,7 +294,7 @@
     <t>Fuse-2920</t>
   </si>
   <si>
-    <t>DC-003A-3.5A-1.3</t>
+    <t>DC-044K-D025</t>
   </si>
   <si>
     <t>S5B-XH-A(LF)(SN)</t>
@@ -342,6 +342,9 @@
     <t>GRM21BR61A226ME44L</t>
   </si>
   <si>
+    <t>CC0603JRX7R9BB104</t>
+  </si>
+  <si>
     <t>GCM21BC72A105KE36L</t>
   </si>
   <si>
@@ -396,6 +399,9 @@
     <t>RC0402FR-074K7L</t>
   </si>
   <si>
+    <t>51R 1W</t>
+  </si>
+  <si>
     <t>RC0402FR-0710KL</t>
   </si>
   <si>
@@ -438,7 +444,7 @@
     <t>BHFUSE</t>
   </si>
   <si>
-    <t>XKB Connection</t>
+    <t>G-Switch</t>
   </si>
   <si>
     <t>BOOMELE</t>
@@ -531,15 +537,12 @@
     <t>Value</t>
   </si>
   <si>
+    <t>Module</t>
+  </si>
+  <si>
     <t>https://fr.aliexpress.com/item/1005004709078383.html?spm=a2g0o.productlist.main.57.6d95f397cf7gmb&amp;algo_pvid=edcdcb7e-db68-42b8-a831-237760419952&amp;algo_exp_id=edcdcb7e-db68-42b8-a831-237760419952-</t>
   </si>
   <si>
-    <t>Module</t>
-  </si>
-  <si>
-    <t>51R 1W (Custom)</t>
-  </si>
-  <si>
     <t>-</t>
   </si>
   <si>
@@ -549,13 +552,7 @@
     <t>SMB</t>
   </si>
   <si>
-    <t>SMB (DO-214AA)</t>
-  </si>
-  <si>
-    <t>CC0603JRX7R9BB104</t>
-  </si>
-  <si>
-    <t>CAP CER 0.1UF 50V X7R 0603</t>
+    <t>SMB(DO-214AA)</t>
   </si>
 </sst>
 </file>
@@ -767,11 +764,11 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="6" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1062,21 +1059,21 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:K35"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="3.109375" style="4" customWidth="1"/>
-    <col min="3" max="3" width="18.6640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="3.140625" style="4" customWidth="1"/>
+    <col min="3" max="3" width="18.7109375" style="4" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="36" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="30" customWidth="1"/>
-    <col min="6" max="6" width="26.5546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="33.44140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="21.44140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="17.88671875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="16.6640625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="29.44140625" customWidth="1"/>
+    <col min="6" max="6" width="26.5703125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="33.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="21.42578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="17.85546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="16.7109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="29.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1"/>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -1085,11 +1082,11 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
-      <c r="I1" s="15"/>
-      <c r="J1" s="15"/>
-      <c r="K1" s="15"/>
-    </row>
-    <row r="2" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="I1" s="14"/>
+      <c r="J1" s="14"/>
+      <c r="K1" s="14"/>
+    </row>
+    <row r="2" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
       <c r="B2" s="5" t="s">
         <v>0</v>
@@ -1098,10 +1095,10 @@
         <v>1</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="F2" s="5" t="s">
         <v>83</v>
@@ -1110,19 +1107,19 @@
         <v>104</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="I2" s="6" t="s">
+        <v>171</v>
+      </c>
+      <c r="J2" s="5" t="s">
         <v>169</v>
       </c>
-      <c r="J2" s="5" t="s">
-        <v>167</v>
-      </c>
       <c r="K2" s="5" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1"/>
       <c r="B3" s="11">
         <f>ROW(B3) - ROW($B$2)</f>
@@ -1132,10 +1129,10 @@
         <v>2</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="F3" s="7" t="s">
         <v>84</v>
@@ -1144,17 +1141,17 @@
         <v>105</v>
       </c>
       <c r="H3" s="7" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="I3" s="8" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="J3" s="7">
         <v>2</v>
       </c>
       <c r="K3" s="7"/>
     </row>
-    <row r="4" spans="1:11" ht="36.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1"/>
       <c r="B4" s="11">
         <f t="shared" ref="B4:B34" si="0">ROW(B4) - ROW($B$2)</f>
@@ -1164,29 +1161,29 @@
         <v>2</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E4" s="10" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="G4" s="10" t="s">
         <v>85</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="I4" s="10" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="J4" s="9">
         <v>2</v>
       </c>
       <c r="K4" s="9"/>
     </row>
-    <row r="5" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1"/>
       <c r="B5" s="11">
         <f>ROW(B5) - ROW($B$2)</f>
@@ -1196,10 +1193,10 @@
         <v>2</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F5" s="7" t="s">
         <v>86</v>
@@ -1208,17 +1205,17 @@
         <v>106</v>
       </c>
       <c r="H5" s="7" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="I5" s="8" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="J5" s="7">
         <v>3</v>
       </c>
       <c r="K5" s="7"/>
     </row>
-    <row r="6" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="1"/>
       <c r="B6" s="11">
         <f t="shared" si="0"/>
@@ -1228,29 +1225,29 @@
         <v>2</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E6" s="10" t="s">
-        <v>178</v>
+        <v>53</v>
       </c>
       <c r="F6" s="9" t="s">
         <v>87</v>
       </c>
       <c r="G6" s="10" t="s">
-        <v>177</v>
+        <v>107</v>
       </c>
       <c r="H6" s="9" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="I6" s="10" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="J6" s="9">
         <v>1</v>
       </c>
       <c r="K6" s="9"/>
     </row>
-    <row r="7" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="1"/>
       <c r="B7" s="11">
         <f>ROW(B7) - ROW($B$2)</f>
@@ -1260,7 +1257,7 @@
         <v>2</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E7" s="8" t="s">
         <v>54</v>
@@ -1269,20 +1266,20 @@
         <v>86</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="H7" s="7" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="I7" s="8" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="J7" s="7">
         <v>1</v>
       </c>
       <c r="K7" s="7"/>
     </row>
-    <row r="8" spans="1:11" ht="36.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
       <c r="B8" s="11">
         <f t="shared" si="0"/>
@@ -1292,7 +1289,7 @@
         <v>2</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E8" s="10" t="s">
         <v>55</v>
@@ -1301,20 +1298,20 @@
         <v>88</v>
       </c>
       <c r="G8" s="10" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="H8" s="9" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="I8" s="10" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="J8" s="9">
         <v>1</v>
       </c>
       <c r="K8" s="9"/>
     </row>
-    <row r="9" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
       <c r="B9" s="11">
         <f>ROW(B9) - ROW($B$2)</f>
@@ -1324,7 +1321,7 @@
         <v>2</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E9" s="8" t="s">
         <v>56</v>
@@ -1333,20 +1330,20 @@
         <v>84</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="H9" s="7" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="I9" s="8" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="J9" s="7">
         <v>1</v>
       </c>
       <c r="K9" s="7"/>
     </row>
-    <row r="10" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="1"/>
       <c r="B10" s="11">
         <f t="shared" si="0"/>
@@ -1356,7 +1353,7 @@
         <v>2</v>
       </c>
       <c r="D10" s="9" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E10" s="10" t="s">
         <v>57</v>
@@ -1365,20 +1362,20 @@
         <v>84</v>
       </c>
       <c r="G10" s="10" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="H10" s="9" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="I10" s="10" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="J10" s="9">
         <v>3</v>
       </c>
       <c r="K10" s="9"/>
     </row>
-    <row r="11" spans="1:11" ht="48.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:11" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="1"/>
       <c r="B11" s="11">
         <f>ROW(B11) - ROW($B$2)</f>
@@ -1388,39 +1385,39 @@
         <v>3</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E11" s="8" t="s">
         <v>58</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="G11" s="8" t="s">
         <v>89</v>
       </c>
       <c r="H11" s="7" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="I11" s="8" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="J11" s="7">
         <v>3</v>
       </c>
       <c r="K11" s="7"/>
     </row>
-    <row r="12" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="1"/>
       <c r="B12" s="11">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
       <c r="C12" s="13" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E12" s="10" t="s">
         <v>59</v>
@@ -1429,20 +1426,20 @@
         <v>88</v>
       </c>
       <c r="G12" s="10" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="H12" s="9" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="I12" s="10" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="J12" s="9">
         <v>1</v>
       </c>
       <c r="K12" s="9"/>
     </row>
-    <row r="13" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="1"/>
       <c r="B13" s="11">
         <f>ROW(B13) - ROW($B$2)</f>
@@ -1452,29 +1449,29 @@
         <v>4</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E13" s="8" t="s">
         <v>60</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="G13" s="8" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="H13" s="7" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="I13" s="8" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="J13" s="7">
         <v>1</v>
       </c>
       <c r="K13" s="7"/>
     </row>
-    <row r="14" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="1"/>
       <c r="B14" s="11">
         <f t="shared" si="0"/>
@@ -1484,29 +1481,29 @@
         <v>4</v>
       </c>
       <c r="D14" s="9" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E14" s="10" t="s">
         <v>61</v>
       </c>
       <c r="F14" s="9" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="G14" s="10" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="H14" s="9" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="I14" s="10" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="J14" s="9">
         <v>1</v>
       </c>
       <c r="K14" s="9"/>
     </row>
-    <row r="15" spans="1:11" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="1"/>
       <c r="B15" s="11">
         <f>ROW(B15) - ROW($B$2)</f>
@@ -1516,7 +1513,7 @@
         <v>5</v>
       </c>
       <c r="D15" s="7" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E15" s="8" t="s">
         <v>62</v>
@@ -1525,20 +1522,20 @@
         <v>90</v>
       </c>
       <c r="G15" s="8" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="H15" s="7" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="I15" s="8" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="J15" s="7">
         <v>2</v>
       </c>
       <c r="K15" s="7"/>
     </row>
-    <row r="16" spans="1:11" ht="36.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="1"/>
       <c r="B16" s="11">
         <f t="shared" si="0"/>
@@ -1548,29 +1545,29 @@
         <v>6</v>
       </c>
       <c r="D16" s="9" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E16" s="10" t="s">
         <v>63</v>
       </c>
       <c r="F16" s="9" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="G16" s="10" t="s">
         <v>91</v>
       </c>
       <c r="H16" s="9" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="I16" s="10" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="J16" s="9">
         <v>1</v>
       </c>
       <c r="K16" s="9"/>
     </row>
-    <row r="17" spans="1:11" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="1"/>
       <c r="B17" s="11">
         <f>ROW(B17) - ROW($B$2)</f>
@@ -1580,61 +1577,61 @@
         <v>6</v>
       </c>
       <c r="D17" s="7" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E17" s="8" t="s">
         <v>64</v>
       </c>
       <c r="F17" s="9" t="s">
+        <v>175</v>
+      </c>
+      <c r="G17" s="8" t="s">
+        <v>116</v>
+      </c>
+      <c r="H17" s="7" t="s">
+        <v>142</v>
+      </c>
+      <c r="I17" s="8" t="s">
         <v>174</v>
-      </c>
-      <c r="G17" s="8" t="s">
-        <v>115</v>
-      </c>
-      <c r="H17" s="7" t="s">
-        <v>140</v>
-      </c>
-      <c r="I17" s="8" t="s">
-        <v>173</v>
       </c>
       <c r="J17" s="7">
         <v>2</v>
       </c>
       <c r="K17" s="7"/>
     </row>
-    <row r="18" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="1"/>
       <c r="B18" s="11">
         <f t="shared" si="0"/>
         <v>16</v>
       </c>
-      <c r="C18" s="12" t="s">
+      <c r="C18" s="13" t="s">
         <v>6</v>
       </c>
       <c r="D18" s="9" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E18" s="10" t="s">
         <v>65</v>
       </c>
       <c r="F18" s="9" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="G18" s="10" t="s">
         <v>92</v>
       </c>
       <c r="H18" s="9" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="I18" s="10" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="J18" s="9">
         <v>1</v>
       </c>
       <c r="K18" s="9"/>
     </row>
-    <row r="19" spans="1:11" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="1"/>
       <c r="B19" s="11">
         <f>ROW(B19) - ROW($B$2)</f>
@@ -1644,29 +1641,29 @@
         <v>7</v>
       </c>
       <c r="D19" s="7" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E19" s="8" t="s">
         <v>66</v>
       </c>
       <c r="F19" s="9" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="G19" s="8" t="s">
         <v>93</v>
       </c>
       <c r="H19" s="7" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="I19" s="8" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="J19" s="7">
         <v>1</v>
       </c>
       <c r="K19" s="7"/>
     </row>
-    <row r="20" spans="1:11" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="1"/>
       <c r="B20" s="11">
         <f t="shared" si="0"/>
@@ -1676,7 +1673,7 @@
         <v>8</v>
       </c>
       <c r="D20" s="9" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E20" s="10" t="s">
         <v>67</v>
@@ -1685,20 +1682,20 @@
         <v>94</v>
       </c>
       <c r="G20" s="10" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="H20" s="9" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="I20" s="10" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="J20" s="9">
         <v>1</v>
       </c>
       <c r="K20" s="9"/>
     </row>
-    <row r="21" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="1"/>
       <c r="B21" s="11">
         <f>ROW(B21) - ROW($B$2)</f>
@@ -1708,7 +1705,7 @@
         <v>9</v>
       </c>
       <c r="D21" s="7" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E21" s="8" t="s">
         <v>68</v>
@@ -1717,20 +1714,20 @@
         <v>95</v>
       </c>
       <c r="G21" s="8" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="H21" s="7" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="I21" s="8" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="J21" s="7">
         <v>6</v>
       </c>
       <c r="K21" s="7"/>
     </row>
-    <row r="22" spans="1:11" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="1"/>
       <c r="B22" s="11">
         <f t="shared" si="0"/>
@@ -1740,7 +1737,7 @@
         <v>9</v>
       </c>
       <c r="D22" s="9" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E22" s="10" t="s">
         <v>69</v>
@@ -1749,20 +1746,20 @@
         <v>95</v>
       </c>
       <c r="G22" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="H22" s="9" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="I22" s="10" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="J22" s="9">
         <v>3</v>
       </c>
       <c r="K22" s="9"/>
     </row>
-    <row r="23" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="1"/>
       <c r="B23" s="11">
         <f>ROW(B23) - ROW($B$2)</f>
@@ -1772,7 +1769,7 @@
         <v>10</v>
       </c>
       <c r="D23" s="7" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E23" s="8" t="s">
         <v>70</v>
@@ -1781,20 +1778,20 @@
         <v>96</v>
       </c>
       <c r="G23" s="8" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="H23" s="7" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="I23" s="8" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="J23" s="7">
         <v>3</v>
       </c>
       <c r="K23" s="7"/>
     </row>
-    <row r="24" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="1"/>
       <c r="B24" s="11">
         <f t="shared" si="0"/>
@@ -1804,7 +1801,7 @@
         <v>11</v>
       </c>
       <c r="D24" s="9" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E24" s="10" t="s">
         <v>71</v>
@@ -1813,20 +1810,20 @@
         <v>97</v>
       </c>
       <c r="G24" s="10" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="H24" s="9" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="I24" s="10" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="J24" s="9">
         <v>2</v>
       </c>
       <c r="K24" s="9"/>
     </row>
-    <row r="25" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="1"/>
       <c r="B25" s="11">
         <f>ROW(B25) - ROW($B$2)</f>
@@ -1836,7 +1833,7 @@
         <v>11</v>
       </c>
       <c r="D25" s="7" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E25" s="8" t="s">
         <v>72</v>
@@ -1845,30 +1842,30 @@
         <v>98</v>
       </c>
       <c r="G25" s="8" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="H25" s="7" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="I25" s="8" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="J25" s="7">
         <v>4</v>
       </c>
       <c r="K25" s="7"/>
     </row>
-    <row r="26" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="1"/>
       <c r="B26" s="11">
         <f t="shared" si="0"/>
         <v>24</v>
       </c>
       <c r="C26" s="13" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D26" s="9" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E26" s="10" t="s">
         <v>73</v>
@@ -1877,30 +1874,30 @@
         <v>97</v>
       </c>
       <c r="G26" s="10" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="H26" s="9" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="I26" s="10" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="J26" s="9">
         <v>1</v>
       </c>
       <c r="K26" s="9"/>
     </row>
-    <row r="27" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="1"/>
       <c r="B27" s="11">
         <f>ROW(B27) - ROW($B$2)</f>
         <v>25</v>
       </c>
       <c r="C27" s="12" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D27" s="7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E27" s="8" t="s">
         <v>74</v>
@@ -1909,30 +1906,30 @@
         <v>97</v>
       </c>
       <c r="G27" s="8" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="H27" s="7" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="I27" s="8" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="J27" s="7">
         <v>1</v>
       </c>
       <c r="K27" s="7"/>
     </row>
-    <row r="28" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="1"/>
       <c r="B28" s="11">
         <f t="shared" si="0"/>
         <v>26</v>
       </c>
       <c r="C28" s="13" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D28" s="9" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E28" s="10" t="s">
         <v>75</v>
@@ -1941,30 +1938,30 @@
         <v>97</v>
       </c>
       <c r="G28" s="10" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="H28" s="9" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="I28" s="10" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="J28" s="9">
         <v>6</v>
       </c>
       <c r="K28" s="9"/>
     </row>
-    <row r="29" spans="1:11" ht="115.8" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:11" ht="120.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="1"/>
       <c r="B29" s="11">
         <f>ROW(B29) - ROW($B$2)</f>
         <v>27</v>
       </c>
-      <c r="C29" s="12" t="s">
-        <v>12</v>
+      <c r="C29" s="13" t="s">
+        <v>11</v>
       </c>
       <c r="D29" s="7" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E29" s="8" t="s">
         <v>76</v>
@@ -1973,32 +1970,32 @@
         <v>99</v>
       </c>
       <c r="G29" s="8" t="s">
-        <v>172</v>
+        <v>126</v>
       </c>
       <c r="H29" s="7" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="I29" s="8" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="J29" s="7">
         <v>3</v>
       </c>
-      <c r="K29" s="14" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="30" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="K29" s="15" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="1"/>
       <c r="B30" s="11">
         <f t="shared" si="0"/>
         <v>28</v>
       </c>
       <c r="C30" s="13" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D30" s="9" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E30" s="10" t="s">
         <v>77</v>
@@ -2007,62 +2004,62 @@
         <v>97</v>
       </c>
       <c r="G30" s="10" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="H30" s="9" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="I30" s="10" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="J30" s="9">
         <v>3</v>
       </c>
       <c r="K30" s="9"/>
     </row>
-    <row r="31" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="1"/>
       <c r="B31" s="11">
         <f>ROW(B31) - ROW($B$2)</f>
         <v>29</v>
       </c>
       <c r="C31" s="12" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D31" s="7" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E31" s="8" t="s">
         <v>78</v>
       </c>
       <c r="F31" s="7" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="G31" s="8" t="s">
         <v>100</v>
       </c>
       <c r="H31" s="7" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="I31" s="8" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="J31" s="7">
         <v>2</v>
       </c>
       <c r="K31" s="7"/>
     </row>
-    <row r="32" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="1"/>
       <c r="B32" s="11">
         <f t="shared" si="0"/>
         <v>30</v>
       </c>
       <c r="C32" s="13" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D32" s="9" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E32" s="10" t="s">
         <v>79</v>
@@ -2071,30 +2068,30 @@
         <v>101</v>
       </c>
       <c r="G32" s="10" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="H32" s="9" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="I32" s="10" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="J32" s="9">
         <v>1</v>
       </c>
       <c r="K32" s="9"/>
     </row>
-    <row r="33" spans="1:11" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" s="1"/>
       <c r="B33" s="11">
         <f>ROW(B33) - ROW($B$2)</f>
         <v>31</v>
       </c>
       <c r="C33" s="12" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D33" s="7" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E33" s="8" t="s">
         <v>80</v>
@@ -2103,62 +2100,62 @@
         <v>96</v>
       </c>
       <c r="G33" s="8" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="H33" s="7" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="I33" s="8" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="J33" s="7">
         <v>1</v>
       </c>
       <c r="K33" s="7"/>
     </row>
-    <row r="34" spans="1:11" ht="36.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="1"/>
       <c r="B34" s="11">
         <f t="shared" si="0"/>
         <v>32</v>
       </c>
       <c r="C34" s="13" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="D34" s="9" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E34" s="10" t="s">
         <v>81</v>
       </c>
       <c r="F34" s="9" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="G34" s="10" t="s">
         <v>102</v>
       </c>
       <c r="H34" s="9" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="I34" s="10" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="J34" s="9">
         <v>1</v>
       </c>
       <c r="K34" s="9"/>
     </row>
-    <row r="35" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A35" s="1"/>
       <c r="B35" s="11">
         <f>ROW(B35) - ROW($B$2)</f>
         <v>33</v>
       </c>
       <c r="C35" s="12" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D35" s="7" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="E35" s="8" t="s">
         <v>82</v>
@@ -2167,13 +2164,13 @@
         <v>103</v>
       </c>
       <c r="G35" s="8" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="H35" s="7" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="I35" s="8" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="J35" s="7">
         <v>3</v>

</xml_diff>

<commit_message>
#3 51Ohm (R14, R15, R22) Resistor part no updated in Main-Controller-Board, BOM Updated
</commit_message>
<xml_diff>
--- a/Design-Files/Main-Controller-Board-v1.1.0/Deliverables/BOM/Client_BOM_Main-Controller-Board-v1.1.0.xlsx
+++ b/Design-Files/Main-Controller-Board-v1.1.0/Deliverables/BOM/Client_BOM_Main-Controller-Board-v1.1.0.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="242" uniqueCount="178">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="241" uniqueCount="177">
   <si>
     <t>#</t>
   </si>
@@ -399,9 +399,6 @@
     <t>RC0402FR-074K7L</t>
   </si>
   <si>
-    <t>51R 1W</t>
-  </si>
-  <si>
     <t>RC0402FR-0710KL</t>
   </si>
   <si>
@@ -468,9 +465,6 @@
     <t>Nexperia</t>
   </si>
   <si>
-    <t>IBUW</t>
-  </si>
-  <si>
     <t>Omron</t>
   </si>
   <si>
@@ -540,9 +534,6 @@
     <t>Module</t>
   </si>
   <si>
-    <t>https://fr.aliexpress.com/item/1005004709078383.html?spm=a2g0o.productlist.main.57.6d95f397cf7gmb&amp;algo_pvid=edcdcb7e-db68-42b8-a831-237760419952&amp;algo_exp_id=edcdcb7e-db68-42b8-a831-237760419952-</t>
-  </si>
-  <si>
     <t>-</t>
   </si>
   <si>
@@ -553,6 +544,12 @@
   </si>
   <si>
     <t>SMB(DO-214AA)</t>
+  </si>
+  <si>
+    <t>FOJAN</t>
+  </si>
+  <si>
+    <t>FRC2512F51R0TS</t>
   </si>
 </sst>
 </file>
@@ -764,11 +761,11 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="6" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="6" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1082,9 +1079,9 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
-      <c r="I1" s="14"/>
-      <c r="J1" s="14"/>
-      <c r="K1" s="14"/>
+      <c r="I1" s="15"/>
+      <c r="J1" s="15"/>
+      <c r="K1" s="15"/>
     </row>
     <row r="2" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -1107,16 +1104,16 @@
         <v>104</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="I2" s="6" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="J2" s="5" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="K2" s="5" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
     </row>
     <row r="3" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1141,10 +1138,10 @@
         <v>105</v>
       </c>
       <c r="H3" s="7" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="I3" s="8" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="J3" s="7">
         <v>2</v>
@@ -1167,16 +1164,16 @@
         <v>51</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="G4" s="10" t="s">
         <v>85</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="I4" s="10" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="J4" s="9">
         <v>2</v>
@@ -1205,10 +1202,10 @@
         <v>106</v>
       </c>
       <c r="H5" s="7" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="I5" s="8" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="J5" s="7">
         <v>3</v>
@@ -1237,10 +1234,10 @@
         <v>107</v>
       </c>
       <c r="H6" s="9" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="I6" s="10" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="J6" s="9">
         <v>1</v>
@@ -1269,10 +1266,10 @@
         <v>108</v>
       </c>
       <c r="H7" s="7" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="I7" s="8" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="J7" s="7">
         <v>1</v>
@@ -1301,10 +1298,10 @@
         <v>109</v>
       </c>
       <c r="H8" s="9" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="I8" s="10" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="J8" s="9">
         <v>1</v>
@@ -1333,10 +1330,10 @@
         <v>110</v>
       </c>
       <c r="H9" s="7" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="I9" s="8" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="J9" s="7">
         <v>1</v>
@@ -1365,10 +1362,10 @@
         <v>111</v>
       </c>
       <c r="H10" s="9" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="I10" s="10" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="J10" s="9">
         <v>3</v>
@@ -1391,16 +1388,16 @@
         <v>58</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="G11" s="8" t="s">
         <v>89</v>
       </c>
       <c r="H11" s="7" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="I11" s="8" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="J11" s="7">
         <v>3</v>
@@ -1429,10 +1426,10 @@
         <v>112</v>
       </c>
       <c r="H12" s="9" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="I12" s="10" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="J12" s="9">
         <v>1</v>
@@ -1455,16 +1452,16 @@
         <v>60</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="G13" s="8" t="s">
         <v>113</v>
       </c>
       <c r="H13" s="7" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="I13" s="8" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="J13" s="7">
         <v>1</v>
@@ -1487,16 +1484,16 @@
         <v>61</v>
       </c>
       <c r="F14" s="9" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="G14" s="10" t="s">
         <v>114</v>
       </c>
       <c r="H14" s="9" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="I14" s="10" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="J14" s="9">
         <v>1</v>
@@ -1525,10 +1522,10 @@
         <v>115</v>
       </c>
       <c r="H15" s="7" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="I15" s="8" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="J15" s="7">
         <v>2</v>
@@ -1551,16 +1548,16 @@
         <v>63</v>
       </c>
       <c r="F16" s="9" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="G16" s="10" t="s">
         <v>91</v>
       </c>
       <c r="H16" s="9" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="I16" s="10" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="J16" s="9">
         <v>1</v>
@@ -1583,16 +1580,16 @@
         <v>64</v>
       </c>
       <c r="F17" s="9" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="G17" s="8" t="s">
         <v>116</v>
       </c>
       <c r="H17" s="7" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="I17" s="8" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="J17" s="7">
         <v>2</v>
@@ -1615,16 +1612,16 @@
         <v>65</v>
       </c>
       <c r="F18" s="9" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="G18" s="10" t="s">
         <v>92</v>
       </c>
       <c r="H18" s="9" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="I18" s="10" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="J18" s="9">
         <v>1</v>
@@ -1647,16 +1644,16 @@
         <v>66</v>
       </c>
       <c r="F19" s="9" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="G19" s="8" t="s">
         <v>93</v>
       </c>
       <c r="H19" s="7" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="I19" s="8" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="J19" s="7">
         <v>1</v>
@@ -1685,10 +1682,10 @@
         <v>117</v>
       </c>
       <c r="H20" s="9" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="I20" s="10" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="J20" s="9">
         <v>1</v>
@@ -1717,10 +1714,10 @@
         <v>118</v>
       </c>
       <c r="H21" s="7" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="I21" s="8" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="J21" s="7">
         <v>6</v>
@@ -1749,10 +1746,10 @@
         <v>119</v>
       </c>
       <c r="H22" s="9" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="I22" s="10" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="J22" s="9">
         <v>3</v>
@@ -1781,10 +1778,10 @@
         <v>120</v>
       </c>
       <c r="H23" s="7" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="I23" s="8" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="J23" s="7">
         <v>3</v>
@@ -1813,10 +1810,10 @@
         <v>121</v>
       </c>
       <c r="H24" s="9" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="I24" s="10" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="J24" s="9">
         <v>2</v>
@@ -1845,10 +1842,10 @@
         <v>122</v>
       </c>
       <c r="H25" s="7" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="I25" s="8" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="J25" s="7">
         <v>4</v>
@@ -1877,10 +1874,10 @@
         <v>123</v>
       </c>
       <c r="H26" s="9" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="I26" s="10" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="J26" s="9">
         <v>1</v>
@@ -1909,10 +1906,10 @@
         <v>124</v>
       </c>
       <c r="H27" s="7" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="I27" s="8" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="J27" s="7">
         <v>1</v>
@@ -1941,17 +1938,17 @@
         <v>125</v>
       </c>
       <c r="H28" s="9" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="I28" s="10" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="J28" s="9">
         <v>6</v>
       </c>
       <c r="K28" s="9"/>
     </row>
-    <row r="29" spans="1:11" ht="120.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="1"/>
       <c r="B29" s="11">
         <f>ROW(B29) - ROW($B$2)</f>
@@ -1970,20 +1967,18 @@
         <v>99</v>
       </c>
       <c r="G29" s="8" t="s">
-        <v>126</v>
+        <v>176</v>
       </c>
       <c r="H29" s="7" t="s">
-        <v>149</v>
+        <v>175</v>
       </c>
       <c r="I29" s="8" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="J29" s="7">
         <v>3</v>
       </c>
-      <c r="K29" s="15" t="s">
-        <v>173</v>
-      </c>
+      <c r="K29" s="14"/>
     </row>
     <row r="30" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="1"/>
@@ -2004,13 +1999,13 @@
         <v>97</v>
       </c>
       <c r="G30" s="10" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="H30" s="9" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="I30" s="10" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="J30" s="9">
         <v>3</v>
@@ -2033,16 +2028,16 @@
         <v>78</v>
       </c>
       <c r="F31" s="7" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="G31" s="8" t="s">
         <v>100</v>
       </c>
       <c r="H31" s="7" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="I31" s="8" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="J31" s="7">
         <v>2</v>
@@ -2068,13 +2063,13 @@
         <v>101</v>
       </c>
       <c r="G32" s="10" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="H32" s="9" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="I32" s="10" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="J32" s="9">
         <v>1</v>
@@ -2100,13 +2095,13 @@
         <v>96</v>
       </c>
       <c r="G33" s="8" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="H33" s="7" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="I33" s="8" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="J33" s="7">
         <v>1</v>
@@ -2120,7 +2115,7 @@
         <v>32</v>
       </c>
       <c r="C34" s="13" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="D34" s="9" t="s">
         <v>47</v>
@@ -2129,16 +2124,16 @@
         <v>81</v>
       </c>
       <c r="F34" s="9" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="G34" s="10" t="s">
         <v>102</v>
       </c>
       <c r="H34" s="9" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="I34" s="10" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="J34" s="9">
         <v>1</v>
@@ -2164,13 +2159,13 @@
         <v>103</v>
       </c>
       <c r="G35" s="8" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="H35" s="7" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="I35" s="8" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="J35" s="7">
         <v>3</v>
@@ -2181,10 +2176,7 @@
   <mergeCells count="1">
     <mergeCell ref="I1:K1"/>
   </mergeCells>
-  <hyperlinks>
-    <hyperlink ref="K29" r:id="rId1"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId2"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>